<commit_message>
Refactor dsm_scenario.py: single Excel input, no HAZUS coupling, dead code - MA_model_inputs.xlsx is now the only input file; Pop_Data.xlsx no longer read - new Scripts/model_inputs.py loads all parameters from the workbook - new workbook tabs: parameters, occupancy_split, structure_split - removed dead code
</commit_message>
<xml_diff>
--- a/InputData/MA_model_inputs.xlsx
+++ b/InputData/MA_model_inputs.xlsx
@@ -14,6 +14,9 @@
     <sheet name="final pop data" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="final gdp data" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Base_year_values" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="parameters" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="occupancy_split" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="structure_split" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1912,6 +1915,102 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>structure</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>weight</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>LF_wood</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>0.5949847709784617</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Mass_Timber</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>0.0426091162557517</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Steel</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>0.1387693878858432</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>RC</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>0.0458413193439987</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>RM</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>0.0446688405310064</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>URM</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>0.128437116399707</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>MH</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>0.0046894488053042</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -8587,4 +8686,378 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>parameter</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>value</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>unit</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>year_start</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>1997</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>year</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>first year of the dynamic stock model</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>year_end</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>2100</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>year</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>last year of the dynamic stock model</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>base_year</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>2020</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>year</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>calibration year; vintage of the floorspace inventory</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>fa_base_year</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>100.7</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>m2/person</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>MA floorspace per person in the base year</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>area_km2</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>20202</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>km2</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>MA land area, used for population density</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>gamma</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>-0.03</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>population-density exponent (EDGE model)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>beta</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>general GDP elasticity of floor area, pre base year</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>beta_SSP1</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>GDP elasticity after base year, SSP1</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>beta_SSP2</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>GDP elasticity after base year, SSP2</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>beta_SSP3</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>GDP elasticity after base year, SSP3</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>beta_SSP4</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>GDP elasticity after base year, SSP4</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>beta_SSP5</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>1</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>GDP elasticity after base year, SSP5</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>interp_kind</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>cubic</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>scipy interp1d kind for population and GDP</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>occupancy</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>weight</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>res</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>0.724062</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>residential</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>com</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>0.179763</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>commercial</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>pub</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>0.034883</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>public (religious, government, education)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>